<commit_message>
update best perform version
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tinky2026/Documents/code/GeoGNNGraphDetect/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F840BA0-E2BB-F042-A0E8-03634FDFFDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{379C01CA-1A1D-BA40-A389-E26BBCBC003C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-740" yWindow="660" windowWidth="19300" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -79,10 +79,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>all_2l</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Full</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -123,6 +119,10 @@
   </si>
   <si>
     <t>Data</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FullnoReg</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -532,7 +532,7 @@
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>1</v>
@@ -567,49 +567,49 @@
         <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>4</v>
       </c>
       <c r="H2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>19</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>4</v>
       </c>
       <c r="M2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="P2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="5" t="s">
-        <v>19</v>
-      </c>
       <c r="R2" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -645,44 +645,89 @@
     </row>
     <row r="8" spans="1:18">
       <c r="A8" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
+      </c>
+      <c r="B8" s="6">
+        <v>0.74299999999999999</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0.1057</v>
+      </c>
+      <c r="D8" s="6">
+        <v>2.0299999999999999E-2</v>
+      </c>
+      <c r="E8" s="6">
+        <v>3.4700000000000002E-2</v>
+      </c>
+      <c r="F8" s="6">
+        <v>5.2299999999999999E-2</v>
+      </c>
+      <c r="G8" s="7">
+        <v>0.73850000000000005</v>
+      </c>
+      <c r="H8" s="7">
+        <v>8.9599999999999999E-2</v>
+      </c>
+      <c r="I8" s="7">
+        <v>2.3E-2</v>
+      </c>
+      <c r="J8" s="7">
+        <v>3.5900000000000001E-2</v>
+      </c>
+      <c r="K8" s="7">
+        <v>5.1299999999999998E-2</v>
+      </c>
+      <c r="L8" s="8">
+        <v>0.70840000000000003</v>
+      </c>
+      <c r="M8" s="5">
+        <v>6.1800000000000001E-2</v>
+      </c>
+      <c r="N8" s="5">
+        <v>3.8199999999999998E-2</v>
+      </c>
+      <c r="O8" s="5">
+        <v>5.1700000000000003E-2</v>
+      </c>
+      <c r="P8" s="5">
+        <v>5.6300000000000003E-2</v>
       </c>
     </row>
     <row r="9" spans="1:18">
       <c r="A9" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="6">
+        <v>13</v>
+      </c>
+      <c r="B9" s="3">
         <v>0.74039999999999995</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="3">
         <v>0.1033</v>
       </c>
       <c r="D9" s="6">
         <v>2.0299999999999999E-2</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="3">
         <v>3.39E-2</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="3">
         <v>5.0999999999999997E-2</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="4">
         <v>0.73829999999999996</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="4">
         <v>8.3699999999999997E-2</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="4">
         <v>2.2599999999999999E-2</v>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="4">
         <v>3.3599999999999998E-2</v>
       </c>
-      <c r="K9" s="7">
+      <c r="K9" s="4">
         <v>4.7899999999999998E-2</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="5">
         <v>0.70309999999999995</v>
       </c>
       <c r="M9" s="8">
@@ -700,7 +745,7 @@
     </row>
     <row r="10" spans="1:18">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3">
         <v>0.68120000000000003</v>

</xml_diff>

<commit_message>
update code and img
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tinky2026/Documents/code/GeoGNNGraphDetect/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F30338E-A850-EA45-A236-EDE98318C1B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6370F1C5-74B8-D94C-93E7-8978C47653B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="68">
   <si>
     <t>metric</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -319,6 +319,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>MoGEAD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>MMoE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -371,10 +375,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>w/o Orth</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>w/o CE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -388,6 +388,94 @@
   </si>
   <si>
     <t>w/o IMNE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w/o CSR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>商业模拟</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>recall</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="SimSun"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>到的</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>+β</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="SimSun"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>价值</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>recall</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="SimSun"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>的审查成本为</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>γ</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>-0.01γ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ts=269</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ts=456</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ts=154</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>+R*β</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -583,7 +671,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -645,6 +733,13 @@
     <xf numFmtId="176" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="176" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="2" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="2" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="2" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -926,7 +1021,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R46"/>
+  <dimension ref="A1:R52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="26.83203125" style="1" customWidth="1"/>
@@ -957,7 +1052,7 @@
       <c r="J1" s="24"/>
       <c r="K1" s="25"/>
       <c r="L1" s="26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M1" s="27"/>
       <c r="N1" s="27"/>
@@ -1809,7 +1904,7 @@
     </row>
     <row r="25" spans="1:18">
       <c r="A25" s="10" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="B25" s="3">
         <v>0.68120000000000003</v>
@@ -1848,7 +1943,7 @@
         <v>3.5900000000000001E-2</v>
       </c>
       <c r="R25" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:18">
@@ -1892,7 +1987,7 @@
         <v>6.5699999999999995E-2</v>
       </c>
       <c r="R26" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:18">
@@ -1938,7 +2033,7 @@
     </row>
     <row r="28" spans="1:18">
       <c r="A28" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B28" s="6">
         <v>0.75439999999999996</v>
@@ -2201,7 +2296,7 @@
     </row>
     <row r="35" spans="1:18">
       <c r="A35" s="1" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B35" s="3">
         <v>0.74839999999999995</v>
@@ -2242,7 +2337,7 @@
     </row>
     <row r="36" spans="1:18">
       <c r="A36" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B36" s="6">
         <v>0.75439999999999996</v>
@@ -2323,40 +2418,40 @@
       <c r="A39" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B39" s="3">
+      <c r="B39" s="37">
         <v>9.4999999999999998E-3</v>
       </c>
-      <c r="C39" s="3">
+      <c r="C39" s="37">
         <v>2.0500000000000001E-2</v>
       </c>
-      <c r="D39" s="3">
+      <c r="D39" s="37">
         <v>5.21E-2</v>
       </c>
-      <c r="E39" s="3">
+      <c r="E39" s="37">
         <v>9.7699999999999995E-2</v>
       </c>
-      <c r="G39" s="4">
+      <c r="G39" s="37">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="H39" s="4">
+      <c r="H39" s="37">
         <v>1.6400000000000001E-2</v>
       </c>
-      <c r="I39" s="4">
+      <c r="I39" s="37">
         <v>4.7300000000000002E-2</v>
       </c>
-      <c r="J39" s="4">
+      <c r="J39" s="37">
         <v>9.8699999999999996E-2</v>
       </c>
-      <c r="L39" s="5">
+      <c r="L39" s="37">
         <v>9.2999999999999992E-3</v>
       </c>
-      <c r="M39" s="5">
+      <c r="M39" s="37">
         <v>2.1100000000000001E-2</v>
       </c>
-      <c r="N39" s="5">
+      <c r="N39" s="37">
         <v>5.0900000000000001E-2</v>
       </c>
-      <c r="O39" s="12">
+      <c r="O39" s="38">
         <v>9.5000000000000001E-2</v>
       </c>
       <c r="R39" s="14" t="s">
@@ -2529,7 +2624,7 @@
     </row>
     <row r="44" spans="1:18">
       <c r="A44" s="10" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="B44" s="3">
         <v>3.6200000000000003E-2</v>
@@ -2572,82 +2667,117 @@
       <c r="A45" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B45" s="37">
         <v>4.0399999999999998E-2</v>
       </c>
-      <c r="C45" s="3">
+      <c r="C45" s="37">
         <v>9.7900000000000001E-2</v>
       </c>
-      <c r="D45" s="3">
+      <c r="D45" s="37">
         <v>0.18540000000000001</v>
       </c>
-      <c r="E45" s="3">
+      <c r="E45" s="37">
         <v>0.31440000000000001</v>
       </c>
-      <c r="G45" s="4">
+      <c r="G45" s="37">
         <v>3.6600000000000001E-2</v>
       </c>
-      <c r="H45" s="4">
+      <c r="H45" s="37">
         <v>8.43E-2</v>
       </c>
-      <c r="I45" s="4">
+      <c r="I45" s="37">
         <v>0.17530000000000001</v>
       </c>
-      <c r="J45" s="4">
+      <c r="J45" s="37">
         <v>0.30940000000000001</v>
       </c>
-      <c r="L45" s="5">
+      <c r="L45" s="37">
         <v>3.2599999999999997E-2</v>
       </c>
-      <c r="M45" s="5">
+      <c r="M45" s="37">
         <v>7.2099999999999997E-2</v>
       </c>
-      <c r="N45" s="5">
+      <c r="N45" s="37">
         <v>0.12570000000000001</v>
       </c>
-      <c r="O45" s="12">
+      <c r="O45" s="38">
         <v>0.2422</v>
       </c>
     </row>
     <row r="46" spans="1:18">
       <c r="A46" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B46" s="3">
+        <v>44</v>
+      </c>
+      <c r="B46" s="37">
         <v>5.0700000000000002E-2</v>
       </c>
-      <c r="C46" s="6">
+      <c r="C46" s="39">
         <v>0.10920000000000001</v>
       </c>
-      <c r="D46" s="3">
+      <c r="D46" s="37">
         <v>0.21540000000000001</v>
       </c>
-      <c r="E46" s="3">
+      <c r="E46" s="37">
         <v>0.34810000000000002</v>
       </c>
-      <c r="G46" s="4">
+      <c r="G46" s="37">
         <v>4.8099999999999997E-2</v>
       </c>
-      <c r="H46" s="7">
+      <c r="H46" s="39">
         <v>9.1600000000000001E-2</v>
       </c>
-      <c r="I46" s="4">
+      <c r="I46" s="37">
         <v>0.19420000000000001</v>
       </c>
-      <c r="J46" s="4">
+      <c r="J46" s="37">
         <v>0.33169999999999999</v>
       </c>
-      <c r="L46" s="5">
+      <c r="L46" s="37">
         <v>3.8899999999999997E-2</v>
       </c>
-      <c r="M46" s="8">
+      <c r="M46" s="39">
         <v>7.2599999999999998E-2</v>
       </c>
-      <c r="N46" s="5">
+      <c r="N46" s="37">
         <v>0.14249999999999999</v>
       </c>
-      <c r="O46" s="12">
+      <c r="O46" s="38">
         <v>0.26860000000000001</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12">
+      <c r="A49" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B49" s="41" t="s">
+        <v>64</v>
+      </c>
+      <c r="G49" s="42" t="s">
+        <v>65</v>
+      </c>
+      <c r="L49" s="43" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12">
+      <c r="A50" s="40" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12">
+      <c r="A51" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B51" s="41" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12">
+      <c r="A52" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B52" s="41" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2658,6 +2788,7 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -2677,12 +2808,12 @@
         <v>14</v>
       </c>
       <c r="D1" s="29" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="29" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" s="29">
         <v>287195</v>
@@ -2696,7 +2827,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="29" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" s="29">
         <v>408239</v>
@@ -2710,7 +2841,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="29" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B4" s="29">
         <v>405543</v>
@@ -2724,7 +2855,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="29" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B5" s="29">
         <v>2696</v>
@@ -2767,7 +2898,7 @@
       <c r="H17" s="33"/>
       <c r="I17" s="33"/>
       <c r="J17" s="33" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K17" s="33"/>
       <c r="L17" s="33"/>
@@ -2775,40 +2906,40 @@
     </row>
     <row r="18" spans="1:13" ht="16">
       <c r="A18" s="32" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B18" s="34" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C18" s="34" t="s">
         <v>5</v>
       </c>
       <c r="D18" s="35" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E18" s="34" t="s">
         <v>7</v>
       </c>
       <c r="F18" s="34" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G18" s="34" t="s">
         <v>5</v>
       </c>
       <c r="H18" s="35" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I18" s="34" t="s">
         <v>7</v>
       </c>
       <c r="J18" s="34" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K18" s="34" t="s">
         <v>5</v>
       </c>
       <c r="L18" s="35" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M18" s="34" t="s">
         <v>7</v>
@@ -3062,7 +3193,7 @@
     </row>
     <row r="25" spans="1:13" ht="16">
       <c r="A25" s="31" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B25" s="34">
         <v>0.68120000000000003</v>
@@ -3185,7 +3316,7 @@
     </row>
     <row r="28" spans="1:13" ht="16">
       <c r="A28" s="31" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B28" s="36">
         <v>0.75439999999999996</v>

</xml_diff>